<commit_message>
[SUPER DUPER Mercury, Venus, Earth, Mars, Jupiter, Saturn, Uranus, and Neptune UPDATE]
</commit_message>
<xml_diff>
--- a/Document/MvA data.xlsx
+++ b/Document/MvA data.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\binhb\Documents\_Unity Projects\Monkey vs Allen\Document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8B65035-007A-4EC9-8A0E-36B791BD0CAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7096115-8DD1-4C39-B871-BA921901E6D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{1F397239-43A2-4385-B6EC-236ED6B8EF51}"/>
   </bookViews>
   <sheets>
     <sheet name="Monkey" sheetId="1" r:id="rId1"/>
-    <sheet name="Tower" sheetId="3" r:id="rId2"/>
-    <sheet name="Allen" sheetId="2" r:id="rId3"/>
-    <sheet name="Player trick" sheetId="4" r:id="rId4"/>
+    <sheet name="MonkeyTower" sheetId="3" r:id="rId2"/>
+    <sheet name="AllenTower" sheetId="5" r:id="rId3"/>
+    <sheet name="Alien" sheetId="2" r:id="rId4"/>
+    <sheet name="Player trick" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="158">
   <si>
     <t>Name</t>
   </si>
@@ -104,9 +105,6 @@
     <t>Vampire</t>
   </si>
   <si>
-    <t>Ném chuối để tấn công</t>
-  </si>
-  <si>
     <t>Bắn tên để tấn công</t>
   </si>
   <si>
@@ -155,9 +153,6 @@
     <t>Mortal</t>
   </si>
   <si>
-    <t>Sniper tower</t>
-  </si>
-  <si>
     <t>"One shot, one kill"</t>
   </si>
   <si>
@@ -215,12 +210,6 @@
     <t>Move speed</t>
   </si>
   <si>
-    <t>Sử dụng lưỡi hái để tấn công</t>
-  </si>
-  <si>
-    <t>Naughty kid</t>
-  </si>
-  <si>
     <t>Knockback</t>
   </si>
   <si>
@@ -317,9 +306,6 @@
     <t>Yorn</t>
   </si>
   <si>
-    <t>Heary</t>
-  </si>
-  <si>
     <t>ArmorII</t>
   </si>
   <si>
@@ -378,6 +364,156 @@
   </si>
   <si>
     <t>Ronin</t>
+  </si>
+  <si>
+    <t>Creed</t>
+  </si>
+  <si>
+    <t>Hayate</t>
+  </si>
+  <si>
+    <t>Ninja</t>
+  </si>
+  <si>
+    <t>BullEye</t>
+  </si>
+  <si>
+    <t>Skill - Shadowstep: Khi kẻ địch đến gần, lập tức tốc biến ra sau, hồi chiêu 10s</t>
+  </si>
+  <si>
+    <t>Skill - Shuriken Toss: Trong 2s, liên tục ném phi tiêu về phía trước. Phi tiêu có khả năng xuyên thấu, mỗi phi tiêu gây 4 sát thương. Tốc đánh càng cao, số phi tiêu càng nhiều. Hồi chiêu 10s. Skill - Shadowstep: Khi kẻ địch đến gần, lập tức tốc biến ra sau, hồi chiêu 10s</t>
+  </si>
+  <si>
+    <t>Tribe</t>
+  </si>
+  <si>
+    <t>Skill - Hashaki: Khi mới sinh ra, nhận hiệu ứng tăng tốc 50% và đòn đánh thường kế tiếp gây thêm 10 sát thương</t>
+  </si>
+  <si>
+    <t>Ưu tiên tấn công kẻ địch ít máu hơn. Ngay lúc sinh ra, nhận hiệu ứng đột kích. Khi giết hoặc hỗ trợ giết kẻ địch, nhận hiệu ứng đột kích</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skill - BountifulHarvest: Giết thành công kẻ địch nhận lại 20% máu đã mất </t>
+  </si>
+  <si>
+    <t>Đòn tấn công gây sát thương lan</t>
+  </si>
+  <si>
+    <t>Ballista</t>
+  </si>
+  <si>
+    <t>Mũi tên đẩy kẻ địch lùi về sau và gây choáng</t>
+  </si>
+  <si>
+    <t>Barret</t>
+  </si>
+  <si>
+    <t>Archmage Tower</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skill - Critical Mass: Sau mỗi 3s nhận một </t>
+  </si>
+  <si>
+    <t>Tower of the Sun</t>
+  </si>
+  <si>
+    <t>Skill - Sun power: Mỗi lần gây sát thương sẽ tích dấu ấn mặt trời lên kẻ địch, kẻ địch nhận tối đa 10 dấu ấn. Mỗi dấu ấn sẽ làm sát thương của Tower này lên mục tiêu đó tăng thêm 1</t>
+  </si>
+  <si>
+    <t>Holy Order</t>
+  </si>
+  <si>
+    <t>Cứ dùng thử đi rồi biết</t>
+  </si>
+  <si>
+    <t>Tiger</t>
+  </si>
+  <si>
+    <t>Chainsaw man</t>
+  </si>
+  <si>
+    <t>Samurai</t>
+  </si>
+  <si>
+    <t>Wu jen</t>
+  </si>
+  <si>
+    <t>Strikethrough</t>
+  </si>
+  <si>
+    <t>JadeEmpire</t>
+  </si>
+  <si>
+    <t>Terracota Warrior</t>
+  </si>
+  <si>
+    <t>Skill - Samurai soul: Khi chết có 15% cơ hội sống thêm 3s nữa và liên tục chém về phía kẻ địch</t>
+  </si>
+  <si>
+    <t>30% Armor; 30% MagicResistance</t>
+  </si>
+  <si>
+    <t>Priestess</t>
+  </si>
+  <si>
+    <t>Skill - Soothe: Hồi 15% máu tối đa và tăng 70% tốc đánh trong 3s. Hồi chiêu 5s</t>
+  </si>
+  <si>
+    <t>Medieval</t>
+  </si>
+  <si>
+    <t>Spearton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GlobalSkill - Shield: Bạn có thể ra lệnh cho Spearton để nó đổi trạng thái: phòng thủ(tăng 30% Armor) hoặc tấn công(tăng 30% tốc đánh) </t>
+  </si>
+  <si>
+    <t>Dropbecon</t>
+  </si>
+  <si>
+    <t>Drop Beacon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cho phép Monkey nhảy dù ở bất cứ vị trí nào trong tháp </t>
+  </si>
+  <si>
+    <t>Tower</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secret Tunnel </t>
+  </si>
+  <si>
+    <t>Altar</t>
+  </si>
+  <si>
+    <t>Skill - Blessing: Toàn bộ Allen nhận được hiệu ứng Momentum trong vòng 3s  khi bắt đầu khởi hành</t>
+  </si>
+  <si>
+    <t>Slingshot master</t>
+  </si>
+  <si>
+    <t>Fennick</t>
+  </si>
+  <si>
+    <t>Skill - Rolling lightning : Kích hoạt khi kẻ địch đến gần, Fennick lộn ra đằng sau 2 ô. Khi nâng cấp sẽ nhận được skill 2 - Sticky bomb: Fennick bắn ra một quả bom khiến kẻ địch chịu hiệu ứng Trói chân trong 5s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sử dụng ná thun để tấn công. </t>
+  </si>
+  <si>
+    <t>Nubby</t>
+  </si>
+  <si>
+    <t>Skill - Alien mask : Monkey này đội mặt nạ để nó trông giống Alien. Alien cứ nghĩ là đồng minh cho đến khi bị Monkey này tấn công</t>
+  </si>
+  <si>
+    <t>Flag Alien</t>
+  </si>
+  <si>
+    <t>Skill - First move: Alien gần nó sẽ nhận được hiệu ứng Momentum</t>
+  </si>
+  <si>
+    <t>Low</t>
   </si>
 </sst>
 </file>
@@ -900,12 +1036,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C2ACF4D6-22E1-47C1-BA3E-E1CA96E3EBAF}" name="Table2" displayName="Table2" ref="A1:K17" totalsRowShown="0">
-  <autoFilter ref="A1:K17" xr:uid="{C2ACF4D6-22E1-47C1-BA3E-E1CA96E3EBAF}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K17">
-    <sortCondition ref="J1:J17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C2ACF4D6-22E1-47C1-BA3E-E1CA96E3EBAF}" name="Table2" displayName="Table2" ref="A1:L32" totalsRowShown="0">
+  <autoFilter ref="A1:L32" xr:uid="{C2ACF4D6-22E1-47C1-BA3E-E1CA96E3EBAF}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L30">
+    <sortCondition ref="K1:K32"/>
   </sortState>
-  <tableColumns count="11">
+  <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{20192834-E586-4E0F-9E8E-718B2BBF9F83}" name="Name"/>
     <tableColumn id="2" xr3:uid="{82E35C8F-4970-42E0-A82E-12588D0E3838}" name="Health"/>
     <tableColumn id="3" xr3:uid="{AE89059C-8518-4487-970D-3902CEE91C8F}" name="Strength"/>
@@ -914,6 +1050,7 @@
     <tableColumn id="10" xr3:uid="{FE0BD48C-193E-4369-A92C-DBE984283068}" name="Move speed"/>
     <tableColumn id="11" xr3:uid="{35579B2B-DCEB-4186-A6A6-03EE29FDADA5}" name="Cooldown"/>
     <tableColumn id="4" xr3:uid="{858A11E4-65AC-4949-82EA-74C2F1BD1C08}" name="Cost"/>
+    <tableColumn id="13" xr3:uid="{D451D5D2-3594-4D63-B952-569D8FED54F1}" name="Tribe"/>
     <tableColumn id="5" xr3:uid="{6DC5BEA6-D16E-4D18-B3C1-F46BA720C2E1}" name="Traits"/>
     <tableColumn id="9" xr3:uid="{9AFCEECD-9C53-4C94-A695-172A1A4EC2FE}" name="Role"/>
     <tableColumn id="6" xr3:uid="{E58DE0E8-2259-4B94-BD3C-FB1FF8F9274F}" name="Description" dataDxfId="25"/>
@@ -923,8 +1060,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5B30ABA4-C722-48F0-950F-D5E600BE35D0}" name="Table5" displayName="Table5" ref="A1:H11" totalsRowShown="0" headerRowDxfId="24" dataDxfId="22" headerRowBorderDxfId="23" tableBorderDxfId="21" totalsRowBorderDxfId="20">
-  <autoFilter ref="A1:H11" xr:uid="{5B30ABA4-C722-48F0-950F-D5E600BE35D0}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5B30ABA4-C722-48F0-950F-D5E600BE35D0}" name="Table5" displayName="Table5" ref="A1:H19" totalsRowShown="0" headerRowDxfId="24" dataDxfId="22" headerRowBorderDxfId="23" tableBorderDxfId="21" totalsRowBorderDxfId="20">
+  <autoFilter ref="A1:H19" xr:uid="{5B30ABA4-C722-48F0-950F-D5E600BE35D0}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{5211774A-CEF8-4106-A5D6-8B4AAC802E93}" name="Name" dataDxfId="19"/>
     <tableColumn id="2" xr3:uid="{E4DC6F0D-D38E-4A33-8EAB-8D2C49E5123E}" name="Health" dataDxfId="18"/>
@@ -941,7 +1078,6 @@
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{226082B9-EAA6-43A4-A488-65E365475C84}" name="Table4" displayName="Table4" ref="A1:J37" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8">
-  <autoFilter ref="A1:J37" xr:uid="{226082B9-EAA6-43A4-A488-65E365475C84}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J37">
     <sortCondition ref="I1:I37"/>
   </sortState>
@@ -1278,16 +1414,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFE84339-B579-4EB3-A65A-1A958D48E7C2}">
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:M30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" customWidth="1"/>
     <col min="3" max="7" width="10.85546875" customWidth="1"/>
-    <col min="9" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="29.140625" style="5" customWidth="1"/>
+    <col min="9" max="9" width="13.28515625" customWidth="1"/>
+    <col min="10" max="10" width="21.7109375" customWidth="1"/>
+    <col min="11" max="11" width="12" customWidth="1"/>
+    <col min="12" max="12" width="32.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1298,13 +1436,13 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" t="s">
         <v>55</v>
-      </c>
-      <c r="E1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F1" t="s">
-        <v>57</v>
       </c>
       <c r="G1" t="s">
         <v>7</v>
@@ -1313,18 +1451,21 @@
         <v>3</v>
       </c>
       <c r="I1" t="s">
+        <v>114</v>
+      </c>
+      <c r="J1" t="s">
         <v>5</v>
       </c>
-      <c r="J1" t="s">
-        <v>65</v>
-      </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" t="s">
+        <v>61</v>
+      </c>
+      <c r="L1" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B2">
         <v>60</v>
@@ -1347,386 +1488,706 @@
       <c r="H2">
         <v>7</v>
       </c>
-      <c r="I2" t="s">
-        <v>43</v>
-      </c>
       <c r="J2" t="s">
-        <v>69</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+      <c r="K2" t="s">
+        <v>65</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>106</v>
-      </c>
-      <c r="J3" t="s">
-        <v>69</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+        <v>101</v>
+      </c>
+      <c r="K3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>109</v>
-      </c>
-      <c r="J4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+      <c r="K4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>137</v>
       </c>
       <c r="B5">
         <v>20</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G5">
         <v>2</v>
       </c>
-      <c r="H5">
-        <v>10</v>
-      </c>
-      <c r="J5" t="s">
-        <v>67</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="L5">
+      <c r="I5" t="s">
+        <v>139</v>
+      </c>
+      <c r="K5" t="s">
+        <v>65</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="M5">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>61</v>
-      </c>
-      <c r="B6">
-        <v>20</v>
-      </c>
-      <c r="C6">
-        <v>8</v>
-      </c>
-      <c r="D6">
-        <v>0.5</v>
-      </c>
-      <c r="E6">
-        <v>6</v>
-      </c>
-      <c r="F6">
-        <v>2</v>
-      </c>
-      <c r="G6">
-        <v>2</v>
-      </c>
-      <c r="H6">
-        <v>10</v>
+        <v>143</v>
       </c>
       <c r="I6" t="s">
-        <v>42</v>
-      </c>
-      <c r="J6" t="s">
-        <v>67</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+      <c r="K6" t="s">
+        <v>65</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>91</v>
+        <v>47</v>
       </c>
       <c r="B7">
         <v>20</v>
       </c>
       <c r="C7">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D7">
         <v>1</v>
       </c>
       <c r="E7">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F7">
         <v>2</v>
       </c>
       <c r="G7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H7">
+        <v>10</v>
+      </c>
+      <c r="K7" t="s">
+        <v>63</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8">
         <v>20</v>
       </c>
-      <c r="J7" t="s">
-        <v>67</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="105" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>105</v>
+      <c r="C8">
+        <v>8</v>
+      </c>
+      <c r="D8">
+        <v>0.5</v>
+      </c>
+      <c r="E8">
+        <v>6</v>
+      </c>
+      <c r="F8">
+        <v>2</v>
+      </c>
+      <c r="G8">
+        <v>2</v>
+      </c>
+      <c r="H8">
+        <v>10</v>
       </c>
       <c r="J8" t="s">
-        <v>67</v>
-      </c>
-      <c r="K8" s="5" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="K8" t="s">
+        <v>63</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>112</v>
+        <v>87</v>
       </c>
       <c r="B9">
         <v>20</v>
       </c>
       <c r="C9">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9">
+        <v>7</v>
+      </c>
+      <c r="F9">
+        <v>2</v>
+      </c>
+      <c r="G9">
+        <v>3</v>
+      </c>
+      <c r="H9">
+        <v>20</v>
+      </c>
+      <c r="K9" t="s">
+        <v>63</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="90" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>100</v>
+      </c>
+      <c r="K10" t="s">
+        <v>63</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>129</v>
+      </c>
+      <c r="B11">
+        <v>10</v>
+      </c>
+      <c r="C11">
+        <v>3</v>
+      </c>
+      <c r="D11">
+        <v>4</v>
+      </c>
+      <c r="E11">
         <v>1.5</v>
       </c>
-      <c r="F9">
+      <c r="F11">
+        <v>2</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="K11" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>149</v>
+      </c>
+      <c r="B12">
+        <v>12</v>
+      </c>
+      <c r="C12">
         <v>3</v>
       </c>
-      <c r="G9">
-        <v>2</v>
-      </c>
-      <c r="J9" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>47</v>
-      </c>
-      <c r="B10">
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>4</v>
+      </c>
+      <c r="F12">
+        <v>3</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12">
+        <v>5</v>
+      </c>
+      <c r="K12" t="s">
+        <v>63</v>
+      </c>
+      <c r="L12" s="5" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13">
         <v>200</v>
       </c>
-      <c r="C10">
+      <c r="C13">
         <v>6</v>
       </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-      <c r="E10">
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
         <v>1.5</v>
       </c>
-      <c r="F10">
-        <v>1</v>
-      </c>
-      <c r="G10">
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13">
         <v>3</v>
       </c>
-      <c r="H10">
+      <c r="H13">
         <v>15</v>
       </c>
-      <c r="I10" t="s">
-        <v>60</v>
-      </c>
-      <c r="J10" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11">
+      <c r="J13" t="s">
+        <v>56</v>
+      </c>
+      <c r="K13" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14">
         <v>140</v>
       </c>
-      <c r="C11">
+      <c r="C14">
         <v>10</v>
       </c>
-      <c r="D11">
+      <c r="D14">
         <v>0.2</v>
       </c>
-      <c r="E11">
+      <c r="E14">
         <v>9</v>
       </c>
-      <c r="F11">
-        <v>1</v>
-      </c>
-      <c r="G11">
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
         <v>3</v>
       </c>
-      <c r="H11">
+      <c r="H14">
         <v>5</v>
       </c>
-      <c r="I11" t="s">
-        <v>42</v>
-      </c>
-      <c r="J11" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>53</v>
-      </c>
-      <c r="B12">
+      <c r="J14" t="s">
         <v>40</v>
       </c>
-      <c r="C12">
+      <c r="K14" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15">
+        <v>40</v>
+      </c>
+      <c r="C15">
         <v>4</v>
       </c>
-      <c r="D12">
-        <v>1</v>
-      </c>
-      <c r="E12">
-        <v>1</v>
-      </c>
-      <c r="F12">
-        <v>2</v>
-      </c>
-      <c r="G12">
-        <v>2</v>
-      </c>
-      <c r="H12">
-        <v>7</v>
-      </c>
-      <c r="J12" t="s">
-        <v>66</v>
-      </c>
-      <c r="K12" s="5" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="75" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>110</v>
-      </c>
-      <c r="B13">
-        <v>80</v>
-      </c>
-      <c r="J13" t="s">
-        <v>66</v>
-      </c>
-      <c r="K13" s="5" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>54</v>
-      </c>
-      <c r="B14">
-        <v>20</v>
-      </c>
-      <c r="C14">
-        <v>3</v>
-      </c>
-      <c r="D14">
-        <v>1</v>
-      </c>
-      <c r="E14">
-        <v>1</v>
-      </c>
-      <c r="F14">
-        <v>2</v>
-      </c>
-      <c r="G14">
-        <v>1</v>
-      </c>
-      <c r="H14">
-        <v>3</v>
-      </c>
-      <c r="J14" t="s">
-        <v>92</v>
-      </c>
-      <c r="K14" s="5" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B15">
-        <v>20</v>
-      </c>
-      <c r="C15">
-        <v>6</v>
-      </c>
       <c r="D15">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E15">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="F15">
         <v>2</v>
       </c>
       <c r="G15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H15">
-        <v>6</v>
-      </c>
-      <c r="J15" t="s">
-        <v>68</v>
-      </c>
-      <c r="K15" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="K15" t="s">
+        <v>62</v>
+      </c>
+      <c r="L15" s="5" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>59</v>
+        <v>105</v>
       </c>
       <c r="B16">
-        <v>10</v>
-      </c>
-      <c r="C16">
-        <v>2</v>
-      </c>
-      <c r="D16">
-        <v>1.5</v>
-      </c>
-      <c r="E16">
-        <v>5</v>
-      </c>
-      <c r="F16">
-        <v>3</v>
-      </c>
-      <c r="G16">
-        <v>1</v>
-      </c>
-      <c r="H16">
-        <v>5</v>
-      </c>
-      <c r="J16" t="s">
-        <v>68</v>
-      </c>
-      <c r="K16" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+      <c r="K16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L16" s="5" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>52</v>
       </c>
+      <c r="B17">
+        <v>20</v>
+      </c>
+      <c r="C17">
+        <v>3</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
       <c r="F17">
         <v>2</v>
+      </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
+        <v>3</v>
+      </c>
+      <c r="K17" t="s">
+        <v>62</v>
+      </c>
+      <c r="L17" s="5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>128</v>
+      </c>
+      <c r="I18" t="s">
+        <v>133</v>
+      </c>
+      <c r="K18" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>130</v>
+      </c>
+      <c r="B19">
+        <v>30</v>
+      </c>
+      <c r="C19">
+        <v>8</v>
+      </c>
+      <c r="D19">
+        <v>0.5</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19">
+        <v>2</v>
+      </c>
+      <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19">
+        <v>6</v>
+      </c>
+      <c r="I19" t="s">
+        <v>133</v>
+      </c>
+      <c r="J19" t="s">
+        <v>111</v>
+      </c>
+      <c r="K19" t="s">
+        <v>62</v>
+      </c>
+      <c r="L19" s="5" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>134</v>
+      </c>
+      <c r="B20">
+        <v>60</v>
+      </c>
+      <c r="C20">
+        <v>8</v>
+      </c>
+      <c r="D20">
+        <v>0.5</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20">
+        <v>2</v>
+      </c>
+      <c r="I20" t="s">
+        <v>133</v>
+      </c>
+      <c r="J20" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="K20" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>140</v>
+      </c>
+      <c r="I21" t="s">
+        <v>139</v>
+      </c>
+      <c r="K21" t="s">
+        <v>62</v>
+      </c>
+      <c r="L21" s="5" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>6</v>
+      </c>
+      <c r="B22">
+        <v>20</v>
+      </c>
+      <c r="C22">
+        <v>6</v>
+      </c>
+      <c r="D22">
+        <v>0.5</v>
+      </c>
+      <c r="E22">
+        <v>9</v>
+      </c>
+      <c r="F22">
+        <v>2</v>
+      </c>
+      <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22">
+        <v>6</v>
+      </c>
+      <c r="K22" t="s">
+        <v>64</v>
+      </c>
+      <c r="L22" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>108</v>
+      </c>
+      <c r="K23" t="s">
+        <v>64</v>
+      </c>
+      <c r="L23" s="5" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" ht="120" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>109</v>
+      </c>
+      <c r="B24">
+        <v>20</v>
+      </c>
+      <c r="E24">
+        <v>5</v>
+      </c>
+      <c r="F24">
+        <v>3</v>
+      </c>
+      <c r="G24">
+        <v>3</v>
+      </c>
+      <c r="H24">
+        <v>15</v>
+      </c>
+      <c r="I24" t="s">
+        <v>133</v>
+      </c>
+      <c r="J24" t="s">
+        <v>111</v>
+      </c>
+      <c r="K24" t="s">
+        <v>64</v>
+      </c>
+      <c r="L24" s="5" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>110</v>
+      </c>
+      <c r="B25">
+        <v>20</v>
+      </c>
+      <c r="C25">
+        <v>3</v>
+      </c>
+      <c r="E25">
+        <v>5</v>
+      </c>
+      <c r="F25">
+        <v>3</v>
+      </c>
+      <c r="G25">
+        <v>1</v>
+      </c>
+      <c r="H25">
+        <v>10</v>
+      </c>
+      <c r="I25" t="s">
+        <v>133</v>
+      </c>
+      <c r="J25" t="s">
+        <v>111</v>
+      </c>
+      <c r="K25" t="s">
+        <v>64</v>
+      </c>
+      <c r="L25" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>50</v>
+      </c>
+      <c r="F26">
+        <v>2</v>
+      </c>
+      <c r="K26" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>107</v>
+      </c>
+      <c r="B27">
+        <v>20</v>
+      </c>
+      <c r="C27">
+        <v>8</v>
+      </c>
+      <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27">
+        <v>1.5</v>
+      </c>
+      <c r="F27">
+        <v>3</v>
+      </c>
+      <c r="G27">
+        <v>2</v>
+      </c>
+      <c r="K27" t="s">
+        <v>64</v>
+      </c>
+      <c r="L27" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>131</v>
+      </c>
+      <c r="B28">
+        <v>20</v>
+      </c>
+      <c r="C28">
+        <v>3</v>
+      </c>
+      <c r="D28">
+        <v>0.5</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="G28">
+        <v>2</v>
+      </c>
+      <c r="I28" t="s">
+        <v>133</v>
+      </c>
+      <c r="J28" t="s">
+        <v>132</v>
+      </c>
+      <c r="K28" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>150</v>
+      </c>
+      <c r="B29">
+        <v>20</v>
+      </c>
+      <c r="C29">
+        <v>4</v>
+      </c>
+      <c r="D29">
+        <v>1.5</v>
+      </c>
+      <c r="E29">
+        <v>5</v>
+      </c>
+      <c r="K29" t="s">
+        <v>64</v>
+      </c>
+      <c r="L29" s="5" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>153</v>
+      </c>
+      <c r="B30">
+        <v>20</v>
+      </c>
+      <c r="K30" t="s">
+        <v>64</v>
+      </c>
+      <c r="L30" s="5" t="s">
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -1739,13 +2200,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBF7BA20-BB6F-4C8E-925E-ECE86D2D9DB6}">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
     <col min="3" max="3" width="10.85546875" customWidth="1"/>
     <col min="4" max="4" width="14.7109375" customWidth="1"/>
-    <col min="8" max="8" width="27.140625" customWidth="1"/>
+    <col min="8" max="8" width="44.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -1759,10 +2220,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>3</v>
@@ -1776,7 +2237,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1788,7 +2249,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -1800,7 +2261,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -1808,13 +2269,13 @@
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H4" s="8"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>38</v>
+        <v>121</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -1823,12 +2284,12 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -1837,12 +2298,12 @@
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
       <c r="H6" s="8" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -1853,44 +2314,146 @@
       <c r="H7" s="9"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
+      <c r="A8" s="1" t="s">
+        <v>36</v>
+      </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
-      <c r="H8" s="8"/>
+      <c r="H8" s="8" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
+      <c r="A9" s="2" t="s">
+        <v>119</v>
+      </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
-      <c r="H9" s="9"/>
+      <c r="H9" s="9" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
+      <c r="A10" s="1" t="s">
+        <v>122</v>
+      </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
-      <c r="H10" s="8"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="11"/>
+      <c r="H10" s="8" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" s="11" t="s">
+        <v>124</v>
+      </c>
       <c r="B11" s="11"/>
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
       <c r="E11" s="11"/>
       <c r="F11" s="11"/>
       <c r="G11" s="11"/>
-      <c r="H11" s="12"/>
+      <c r="H11" s="12" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="9" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="9"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="9"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="9"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="9"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="9"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="9"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1901,6 +2464,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{879C6548-91A9-48A8-8FC9-F010852558EA}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E85F11D4-018E-41F8-95AA-DA05607C5C9A}">
   <dimension ref="A1:K39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1936,16 +2508,16 @@
         <v>5</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="J1" s="7" t="s">
         <v>4</v>
       </c>
       <c r="K1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -1968,10 +2540,10 @@
         <v>60</v>
       </c>
       <c r="G2" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="I2" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>17</v>
@@ -1988,61 +2560,61 @@
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E4">
         <v>10</v>
       </c>
       <c r="I4" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E5">
         <v>25</v>
       </c>
       <c r="G5" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H5" t="s">
         <v>11</v>
       </c>
       <c r="I5" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="G6" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="I6" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -2062,10 +2634,10 @@
         <v>30</v>
       </c>
       <c r="I7" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -2082,7 +2654,7 @@
         <v>1</v>
       </c>
       <c r="I8" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2102,10 +2674,10 @@
         <v>30</v>
       </c>
       <c r="I9" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="K9">
         <v>2</v>
@@ -2128,13 +2700,13 @@
         <v>60</v>
       </c>
       <c r="G10" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I10" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -2148,21 +2720,21 @@
         <v>0</v>
       </c>
       <c r="G11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I11" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B12">
         <v>60</v>
@@ -2174,26 +2746,26 @@
         <v>1</v>
       </c>
       <c r="I12" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="H13" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="I13" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B14">
         <v>80</v>
@@ -2205,13 +2777,13 @@
         <v>1</v>
       </c>
       <c r="G14" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="H14" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="I14" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -2234,12 +2806,12 @@
         <v>11</v>
       </c>
       <c r="I15" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B16">
         <v>140</v>
@@ -2254,15 +2826,15 @@
         <v>60</v>
       </c>
       <c r="I16" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B17">
         <v>60</v>
@@ -2274,15 +2846,15 @@
         <v>1</v>
       </c>
       <c r="G17" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="I17" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B18">
         <v>20</v>
@@ -2291,29 +2863,29 @@
         <v>3</v>
       </c>
       <c r="I18" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B19">
         <v>20</v>
       </c>
       <c r="I19" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B20">
         <v>120</v>
@@ -2322,12 +2894,12 @@
         <v>2</v>
       </c>
       <c r="I20" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B21">
         <v>20</v>
@@ -2342,12 +2914,12 @@
         <v>7</v>
       </c>
       <c r="I21" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B22">
         <v>20</v>
@@ -2362,15 +2934,15 @@
         <v>-1</v>
       </c>
       <c r="I22" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B23">
         <v>60</v>
@@ -2382,7 +2954,7 @@
         <v>1</v>
       </c>
       <c r="I23" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -2402,7 +2974,7 @@
         <v>5</v>
       </c>
       <c r="I24" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="J24" s="5" t="s">
         <v>18</v>
@@ -2410,43 +2982,91 @@
     </row>
     <row r="25" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="I25" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="G26" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="I26" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="H27" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="I27" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>101</v>
+        <v>96</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>147</v>
+      </c>
+      <c r="E30">
+        <v>15</v>
+      </c>
+      <c r="H30" t="s">
+        <v>145</v>
+      </c>
+      <c r="I30" t="s">
+        <v>65</v>
+      </c>
+      <c r="J30" s="5" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>155</v>
+      </c>
+      <c r="B31">
+        <v>300</v>
+      </c>
+      <c r="C31">
+        <v>30</v>
+      </c>
+      <c r="D31">
+        <v>2</v>
+      </c>
+      <c r="E31">
+        <v>6</v>
+      </c>
+      <c r="F31" t="s">
+        <v>157</v>
+      </c>
+      <c r="I31" t="s">
+        <v>65</v>
+      </c>
+      <c r="J31" s="5" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="37" spans="3:3" x14ac:dyDescent="0.25">
@@ -2463,7 +3083,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A53618B-D135-4ACB-A136-E1671DC87E69}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2473,6 +3093,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="8428bf46-4a85-4a22-93bf-eed677f88aa1" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Tài liệu" ma:contentTypeID="0x010100B0D00C5572DCC04391B215DBDA0093DE" ma:contentTypeVersion="12" ma:contentTypeDescription="Tạo tài liệu mới." ma:contentTypeScope="" ma:versionID="b78c5497871d53d1071afebf040bf691">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="8428bf46-4a85-4a22-93bf-eed677f88aa1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="80b18ca4aec3b99efe8c6501d055a54a" ns3:_="">
     <xsd:import namespace="8428bf46-4a85-4a22-93bf-eed677f88aa1"/>
@@ -2666,24 +3303,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D7A71F8-F801-477D-88A9-C0850BF52685}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="8428bf46-4a85-4a22-93bf-eed677f88aa1"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="8428bf46-4a85-4a22-93bf-eed677f88aa1" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{996EA4C5-F47F-49CB-AE30-AC01B68D77DB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A9506F2-3473-4062-8CC1-60D3A3FAEA8D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2699,28 +3343,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{996EA4C5-F47F-49CB-AE30-AC01B68D77DB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D7A71F8-F801-477D-88A9-C0850BF52685}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="8428bf46-4a85-4a22-93bf-eed677f88aa1"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>